<commit_message>
fix(capmatrix): preserve the required capability names exactly (rows 20/33/40)
The first publication rendered three capability names with ASCII arrows
('<->', '->') instead of the required '↔' and '→'. Post-merge independent
retrieval caught it: rows 20, 33 and 40 did not match the required inventory
verbatim. Names corrected; report, CSV and XLSX regenerated from the single
data source; no status value changed.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/evidence/cross-repository/artifacts/IIPS_V3_CAPABILITY_MATRIX_51x17_2026-10-23.xlsx
+++ b/evidence/cross-repository/artifacts/IIPS_V3_CAPABILITY_MATRIX_51x17_2026-10-23.xlsx
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>PIT read seam + `/api/pit/market-data` (IRR &lt;-&gt; IPD, Gate 43)</t>
+          <t>PIT read seam + `/api/pit/market-data` (IRR ↔ IPD, Gate 43)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Owner-&gt;G24 binding chain `P-2` -&gt; `P-4` -&gt; `P-6` -&gt; `P-8` (IRR + IPD)</t>
+          <t>Owner→G24 binding chain `P-2` → `P-4` → `P-6` → `P-8` (IRR + IPD)</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Certified-analytics &lt;-&gt; user-portfolio integration</t>
+          <t>Certified-analytics ↔ user-portfolio integration</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">

</xml_diff>